<commit_message>
Updated ARE_grids_kan model - 2026-03-03 16:37
</commit_message>
<xml_diff>
--- a/VerveStacks_ARE_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ARE_grids_kan/ReportDefs_vervestacks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ARE_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{789ADFF8-066D-4A61-8BA6-83EF99E5DE82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F419421F-CCC0-4958-9834-B1CE20168315}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3361,7 +3361,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B30D215-4E0A-4A5E-BC8B-2557842FFD65}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{834FEDC3-7D6C-4396-9510-EF1B8FAF8DFB}">
   <dimension ref="B9:H169"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -19606,7 +19606,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D5E2CA4-D52F-4B08-925A-DD06F1903742}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58AB0CAE-315A-4F19-935E-D4E6A80B7911}">
   <dimension ref="B9:L169"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ARE_grids_kan model - 2026-03-10 17:27
</commit_message>
<xml_diff>
--- a/VerveStacks_ARE_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ARE_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ARE_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4A4BE810-F055-4AEC-B65E-EFC9C7A972D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E562AA1F-9492-41A9-8FD2-1BC1C859C6CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3409,7 +3409,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD3178FF-8CED-46E8-9658-1BE80596FCC5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80696747-537C-48D3-97CD-0318089DEE9E}">
   <dimension ref="B9:H169"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -19798,7 +19798,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6122EEEE-5A41-4998-8599-47D862430E5B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21447089-8D33-4793-860F-146478A2F496}">
   <dimension ref="B9:L169"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>